<commit_message>
Remove unused scrape_coconala.py script
Co-authored-by: mail135797 <mail135797@gmail.com>
</commit_message>
<xml_diff>
--- a/labor_shimpan_coconala.xlsx
+++ b/labor_shimpan_coconala.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,22 +453,220 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>吉﨑 眞人弁護士 ベリーベスト法律事務所 奈良オフィス</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://legal.coconala.com/lawyers/4020</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>詳細ページ参照</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Coconala에서 '노동심판' 관련 근로자 측 변호사 서비스를 자동 수집하지 못했습니다. 검색어가 너무 구체적이거나 사이트 구조 변경으로 인한 문제일 수 있습니다.</t>
+          <t>[労働者 / 解雇 / 退職] 電話でお問い合わせ 050-7587-2653 受付中 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:30〜21:00 土日祝日 09:30〜18:00 定休日 なし 定休日補足 2025年12月26日～2026年01月04日 ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>吉村 まどか弁護士 摂津総合法律事務所</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/6175</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[従業員 / 未払い / 解雇] 電話でお問い合わせ 050-7586-2712 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:00〜17:30 定休日 日曜、土曜、祝日 定休日補足 事務所の電話は17:15までとなっております。 以降のご連絡については...</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>山﨑 恒平弁護士 山﨑・新見法律事務所</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/4593</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>[労働者 / 未払い] 電話で面談予約 050-7587-1342 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:30〜18:00 定休日 日曜、土曜、祝日 定休日補足 ※営業時間外の夜間帯でのご相談も日程次第で調整可能です。※メール問い合わせ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>中田 侑佳弁護士 弁護士法人ＯＮＥ 岩国オフィス</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/2193</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>[従業員 / 未払い / 退職] 電話でお問い合わせ 050-7587-2912 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:00〜18:00 定休日 日曜、土曜、祝日 定休日補足 ◆事前予約で当日／夜間/休日相談が対応できる場合があります◆ まずはお...</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>関谷 恵美弁護士 アポロ法律事務所</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/2475</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>[従業員 / 未払い / 退職] 電話でお問い合わせ 050-7587-6895 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:00〜18:00 土日祝日 09:00〜18:00 定休日 日曜、土曜、祝日 定休日補足 メールは24時間対応。法律相談は平日...</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>石濱 貴文弁護士 高松丸亀町法律事務所</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/2341</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>[未払い / 解雇 / 退職] 電話でお問い合わせ 050-7587-0571 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:00〜20:00 定休日 日曜、土曜、祝日 定休日補足 上記時間は、ココナラ法律相談の電話受付時間となり、事務所の営業時間は9...</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>田中 佑樹弁護士 弁護士法人長瀬総合法律事務所 水戸支所</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/1748</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>[労働者] 電話で面談予約 050-7587-8759 定休日 メールで面談予約 ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 06:00〜23:00 土日祝日 06:00〜23:00 定休日 日曜、土曜、祝日 定休日補足 【営業時間】平日09:00-18:00完全予...</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>阪田 裕史弁護士 阪神総合法律事務所</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/4862</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>[従業員 / 未払い / 退職] 電話でお問い合わせ 050-7587-6134 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:30〜17:30 定休日 日曜、土曜、祝日 定休日補足 17:30以降、土日祝日は、事前にご予約いただければご対応可能でござい...</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>中野 公義弁護士 なかのきみよし法律事務所</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/5950</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>[解雇 / パワハラ / セクハラ] 電話で面談予約 050-7586-5884 定休日 メールで面談予約 ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 09:00〜17:00 定休日 日曜、土曜、祝日 定休日補足 事前予約により，出勤前の時間帯（7時30分〜9時）でのご相談も対応いたします。...</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>石井 龍一弁護士 石井法律事務所</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://legal.coconala.com/lawyers/2757</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>詳細ページ参照</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>[未払い] 電話でお問い合わせ 050-7586-3125 定休日 メールでお問い合わせ ※お電話の際は「ココナラ法律相談を見た」とお伝えいただくとスムーズです。 受付時間 平日 00:00〜23:59 土日祝日 00:00〜23:59 定休日 日曜、土曜、祝日 定休日補足 事務所の営業時間は、平日09:00〜...</t>
         </is>
       </c>
     </row>

</xml_diff>